<commit_message>
Update data files - 2026-03-02
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/nifty_options/nifty_options_2026-02.xlsx
+++ b/data/nifty_options/nifty_options_2026-02.xlsx
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE17"/>
+  <dimension ref="A1:AE18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2543,6 +2543,123 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-27</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>10:00:09</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>TRADEABLE</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="6" t="n">
+        <v>25327.45</v>
+      </c>
+      <c r="I18" s="6" t="n">
+        <v>13.54</v>
+      </c>
+      <c r="J18" s="6" t="n">
+        <v>-0.61</v>
+      </c>
+      <c r="K18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="5" t="n">
+        <v>63.1</v>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="N18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T18" s="2" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="U18" s="2" t="inlineStr"/>
+      <c r="V18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC18" s="2" t="inlineStr">
+        <is>
+          <t>HARD VETO: CPR TRENDING DAY: Price 25327.45 below BC 25486.95 - BEARISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AD18" s="2" t="inlineStr">
+        <is>
+          <t>CPR TRENDING DAY: Price 25327.45 below BC 25486.95 - BEARISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AE18" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>